<commit_message>
modularisasi datepicker seems to be done
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -1,64 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7421E32C-7C4A-B34A-845F-8D63A9F64883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>nik</t>
-  </si>
-  <si>
-    <t>nama_lengkap</t>
-  </si>
-  <si>
-    <t>tgl_pemeriksaan</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>3509053001929991</t>
-  </si>
-  <si>
-    <t>Joko</t>
-  </si>
-  <si>
-    <t>2026-05-25</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -77,22 +46,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -412,49 +440,72 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5" bestFit="1" customWidth="1"/>
+    <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.5" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.83203125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="10.83203125" customWidth="1" style="1" min="9" max="9"/>
+    <col width="16" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>nik</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nama_lengkap</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tgl_pemeriksaan</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>3509053001929991</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Joko</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FAILED: Pencarian tidak memberikan hasil atau tombol Konfirmasi Hadir tidak muncul.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add calendar button layout and update registration entry handling
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>3509053001929991</t>
+          <t>3512345598191001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joko</t>
+          <t>Imam Baroroh</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FAILED: Pencarian tidak memberikan hasil atau tombol Konfirmasi Hadir tidak muncul.</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add wait for whatsapp input and handle quota full navigation
- Add 3s wait after filling whatsapp number to ensure UI stability
- Implement try-except block to handle "Quota Penuh" (Quota Full) scenario
- Introduce SkipRowException in custom_exceptions.py to gracefully handle row skipping
- Update main loop to catch SkipRowException and mark rows accordingly
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1800" yWindow="1860" windowWidth="32400" windowHeight="19180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -445,8 +445,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -504,6 +504,300 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>3504016208800001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Siti Nurhamida</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>3512086108860001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Alifa Wulandari</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>3512064301860005</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Amalia</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAILED: Locator.click: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("button:has-text('Konfirmasi Hadir')").first
+    - locator resolved to &lt;button type="button" class="w-fill btn-fill-primary h-11"&gt;…&lt;/button&gt;
+  - attempting click action
+    - waiting for element to be visible, enabled and stable
+  - element was detached from the DOM, retrying
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>3512075610720001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Farah Andriani</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAILED: Locator.click: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("button:has-text('Konfirmasi Hadir')").first
+    - locator resolved to &lt;button type="button" class="w-fill btn-fill-primary h-11"&gt;…&lt;/button&gt;
+  - attempting click action
+    - waiting for element to be visible, enabled and stable
+  - element was detached from the DOM, retrying
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>3512064901750001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Siti Andayani</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>3512076709690002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ary Widjajanti</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>3319091108880005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Masyudi</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>3512096104830001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dwi Usriya</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>3512060209800002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ibnu Haris</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>3512134301930006</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fitri Ayu Nurjannatin</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>3512076508980002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Maya Sukma Indah Refiana</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>3505142311880001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Untung Slamet Setiawan</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>3512074106740002</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Rofiqa Yuni Astuti</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>3512094206710001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Yuni Retnowati</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>3512081110870001</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cahyo Murtanto</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
fix: stage 1 fixing skrining-filtering, change excel file for dewasa
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1800" yWindow="1860" windowWidth="32400" windowHeight="19180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -445,55 +445,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
-    <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
-    <col width="12.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="11.5" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
-    <col width="10.5" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="14.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="10.83203125" customWidth="1" style="1" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="1" min="9" max="9"/>
-    <col width="16" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="13.5" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="12.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10.83203125" customWidth="1" style="1" min="6" max="6"/>
+    <col width="10.83203125" customWidth="1" style="1" min="8" max="8"/>
+    <col width="16" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>nik</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>nama_lengkap</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tgl_pemeriksaan</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Farah Andriani</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Eksan</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Eksan H</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>

</xml_diff>

<commit_message>
fix: stage 9/9 fixing skrining-filtering, excel finalization
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -1,33 +1,61 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9950FA-253D-844A-8545-4F7942F8E812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>nama_lengkap</t>
+  </si>
+  <si>
+    <t>tgl_pemeriksaan</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>BADRI FAUZI</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +74,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -440,78 +409,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="12.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="10.5" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="14.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="10.83203125" customWidth="1" style="1" min="6" max="6"/>
-    <col width="10.83203125" customWidth="1" style="1" min="8" max="8"/>
-    <col width="16" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.5" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>nama_lengkap</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>tgl_pemeriksaan</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Eksan</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Eksan H</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add faker libs
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9950FA-253D-844A-8545-4F7942F8E812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D96DBAE-D522-D046-BFA6-227A7B0BFBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>nama_lengkap</t>
   </si>
@@ -35,9 +35,6 @@
   </si>
   <si>
     <t>2026-07-08</t>
-  </si>
-  <si>
-    <t>SUCCESS</t>
   </si>
 </sst>
 </file>
@@ -442,9 +439,6 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: remove ds store and pengelompokkan.xlsx
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran.xlsx
+++ b/dataset/konfirm_kehadiran.xlsx
@@ -1,58 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D96DBAE-D522-D046-BFA6-227A7B0BFBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>nama_lengkap</t>
-  </si>
-  <si>
-    <t>tgl_pemeriksaan</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>BADRI FAUZI</t>
-  </si>
-  <si>
-    <t>2026-07-08</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -71,22 +46,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -406,42 +440,68 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5" bestFit="1" customWidth="1"/>
+    <col width="25.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10.83203125" customWidth="1" style="1" min="6" max="6"/>
+    <col width="10.83203125" customWidth="1" style="1" min="8" max="8"/>
+    <col width="16" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nama_lengkap</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tgl_pemeriksaan</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BADRI FAUZI</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BADRI FAUZI</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>